<commit_message>
escala HETRIN out/2026: Jaison Correia Costa passa para Noturno ímpar
Linha do Jaison (Aux. Manutenção / Climatização) mudada de NOTURNO PAR para
NOTURNO IMPAR: do dia 8 em diante, N nos dias ímpares e F nos pares (mesmo
padrão e formatação do Manoel Messias). Dias 1–7 seguem em branco (antes do início).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/hetrin/Escala_HETRIN_Outubro_2026.xlsx
+++ b/backend/data/hetrin/Escala_HETRIN_Outubro_2026.xlsx
@@ -2729,7 +2729,7 @@
         <v>50</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>79</v>
@@ -2755,77 +2755,77 @@
       <c r="L22" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="M22" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="N22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="O22" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="P22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q22" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="R22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="S22" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="T22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="U22" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="V22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="W22" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="X22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="Y22" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="Z22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="AA22" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="AB22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="AC22" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="AD22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="AE22" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="AF22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="AG22" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="AH22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="AI22" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="AJ22" s="8" t="s">
-        <v>47</v>
+      <c r="M22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="N22" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="O22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="P22" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="R22" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="S22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="T22" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="U22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="V22" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="W22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="X22" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="Y22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z22" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB22" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AC22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD22" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AE22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF22" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AH22" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AI22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AJ22" s="9" t="s">
+        <v>80</v>
       </c>
       <c r="AK22" s="5" t="s">
         <v>45</v>

</xml_diff>

<commit_message>
feat(hetrin): inclui Natan Nascimento Nunes (Tecnico de Climatizacao, noturno impar, admissao 21/10)
Linha nova na secao NOTURNO da escala de outubro/2026, com plantao (N) so nos dias impares a partir de 21/10
(antes da admissao a celula fica vazia). Edicao direta do XML da planilha para preservar o logo.
Validado: carrega como Tecnico de Climatizacao/Noturno/Ativo e esta disponivel em 21, 23, 25... e nao antes.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/hetrin/Escala_HETRIN_Outubro_2026.xlsx
+++ b/backend/data/hetrin/Escala_HETRIN_Outubro_2026.xlsx
@@ -851,7 +851,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AK33"/>
+  <dimension ref="A1:AK34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -3396,94 +3396,170 @@
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A29" s="10" t="s">
+    <row r="28" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Natan Nascimento Nunes</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Técnico de Climatização</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="M28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="N28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="O28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="P28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="R28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="S28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="T28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="U28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="V28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="W28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="X28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z28" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA28" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB28" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AC28" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD28" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AE28" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF28" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AG28" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AH28" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AI28" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AJ28" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="AK28" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="30" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="10"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="10"/>
-      <c r="L29" s="10"/>
-      <c r="M29" s="10"/>
-      <c r="N29" s="10"/>
-      <c r="O29" s="10"/>
-      <c r="P29" s="10"/>
-      <c r="Q29" s="10"/>
-      <c r="R29" s="10"/>
-      <c r="S29" s="10"/>
-      <c r="T29" s="10"/>
-      <c r="U29" s="10"/>
-      <c r="V29" s="10"/>
-      <c r="W29" s="10"/>
-      <c r="X29" s="10"/>
-      <c r="Y29" s="10"/>
-      <c r="Z29" s="10"/>
-      <c r="AA29" s="10"/>
-      <c r="AB29" s="10"/>
-      <c r="AC29" s="10"/>
-      <c r="AD29" s="10"/>
-      <c r="AE29" s="10"/>
-      <c r="AF29" s="10"/>
-      <c r="AG29" s="10"/>
-      <c r="AH29" s="10"/>
-      <c r="AI29" s="10"/>
-      <c r="AJ29" s="10"/>
-      <c r="AK29" s="10"/>
-    </row>
-    <row r="31" ht="20" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A31" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="B31" s="11"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="11"/>
-      <c r="J31" s="11"/>
-      <c r="K31" s="11"/>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="N31" s="11"/>
-      <c r="O31" s="11"/>
-      <c r="P31" s="11"/>
-      <c r="Q31" s="11"/>
-      <c r="R31" s="11"/>
-      <c r="S31" s="11"/>
-      <c r="T31" s="11"/>
-      <c r="U31" s="11"/>
-      <c r="V31" s="11"/>
-      <c r="W31" s="11"/>
-      <c r="X31" s="11"/>
-      <c r="Y31" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="Z31" s="11"/>
-      <c r="AA31" s="11"/>
-      <c r="AB31" s="11"/>
-      <c r="AC31" s="11"/>
-      <c r="AD31" s="11"/>
-      <c r="AE31" s="11"/>
-      <c r="AF31" s="11"/>
-      <c r="AG31" s="11"/>
-      <c r="AH31" s="11"/>
-      <c r="AI31" s="11"/>
-      <c r="AJ31" s="11"/>
-      <c r="AK31" s="11"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="10"/>
+      <c r="M30" s="10"/>
+      <c r="N30" s="10"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="10"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="10"/>
+      <c r="S30" s="10"/>
+      <c r="T30" s="10"/>
+      <c r="U30" s="10"/>
+      <c r="V30" s="10"/>
+      <c r="W30" s="10"/>
+      <c r="X30" s="10"/>
+      <c r="Y30" s="10"/>
+      <c r="Z30" s="10"/>
+      <c r="AA30" s="10"/>
+      <c r="AB30" s="10"/>
+      <c r="AC30" s="10"/>
+      <c r="AD30" s="10"/>
+      <c r="AE30" s="10"/>
+      <c r="AF30" s="10"/>
+      <c r="AG30" s="10"/>
+      <c r="AH30" s="10"/>
+      <c r="AI30" s="10"/>
+      <c r="AJ30" s="10"/>
+      <c r="AK30" s="10"/>
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A32" s="11"/>
+      <c r="A32" s="11" t="s">
+        <v>98</v>
+      </c>
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
       <c r="D32" s="11"/>
@@ -3495,7 +3571,9 @@
       <c r="J32" s="11"/>
       <c r="K32" s="11"/>
       <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
+      <c r="M32" s="11" t="s">
+        <v>99</v>
+      </c>
       <c r="N32" s="11"/>
       <c r="O32" s="11"/>
       <c r="P32" s="11"/>
@@ -3507,7 +3585,9 @@
       <c r="V32" s="11"/>
       <c r="W32" s="11"/>
       <c r="X32" s="11"/>
-      <c r="Y32" s="11"/>
+      <c r="Y32" s="11" t="s">
+        <v>100</v>
+      </c>
       <c r="Z32" s="11"/>
       <c r="AA32" s="11"/>
       <c r="AB32" s="11"/>
@@ -3560,16 +3640,55 @@
       <c r="AJ33" s="11"/>
       <c r="AK33" s="11"/>
     </row>
+    <row r="34" ht="20" customHeight="1" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="A34" s="11"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="11"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
+      <c r="J34" s="11"/>
+      <c r="K34" s="11"/>
+      <c r="L34" s="11"/>
+      <c r="M34" s="11"/>
+      <c r="N34" s="11"/>
+      <c r="O34" s="11"/>
+      <c r="P34" s="11"/>
+      <c r="Q34" s="11"/>
+      <c r="R34" s="11"/>
+      <c r="S34" s="11"/>
+      <c r="T34" s="11"/>
+      <c r="U34" s="11"/>
+      <c r="V34" s="11"/>
+      <c r="W34" s="11"/>
+      <c r="X34" s="11"/>
+      <c r="Y34" s="11"/>
+      <c r="Z34" s="11"/>
+      <c r="AA34" s="11"/>
+      <c r="AB34" s="11"/>
+      <c r="AC34" s="11"/>
+      <c r="AD34" s="11"/>
+      <c r="AE34" s="11"/>
+      <c r="AF34" s="11"/>
+      <c r="AG34" s="11"/>
+      <c r="AH34" s="11"/>
+      <c r="AI34" s="11"/>
+      <c r="AJ34" s="11"/>
+      <c r="AK34" s="11"/>
+    </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="D1:AK1"/>
     <mergeCell ref="A3:AK3"/>
     <mergeCell ref="A6:AK6"/>
     <mergeCell ref="A18:AK18"/>
-    <mergeCell ref="A29:AK29"/>
-    <mergeCell ref="A31:L33"/>
-    <mergeCell ref="M31:X33"/>
-    <mergeCell ref="Y31:AK33"/>
+    <mergeCell ref="A30:AK30"/>
+    <mergeCell ref="A32:L34"/>
+    <mergeCell ref="M32:X34"/>
+    <mergeCell ref="Y32:AK34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>